<commit_message>
Replace the cabinet descriptions workbook with the newer correction.
Keep the same path and rerun the admin round-trip parser dry run against the updated sheet.

Co-authored-by: 7809tom-sys <7809tom-sys@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/distributor-connections/cabinet-descriptions-corrected-2026-10-26.xlsx
+++ b/data/distributor-connections/cabinet-descriptions-corrected-2026-10-26.xlsx
@@ -190,6 +190,41 @@
     <author>Grok Bot</author>
   </authors>
   <commentList>
+    <comment ref="B86" authorId="0" shapeId="0">
+      <text>
+        <t>42" diagonal corner sink base: the front/side piece (DCSF42, row 234) and the bottom/floor piece (SBF4242, row 86) must be purchased together; DCFF42 (row 232) is the combined front &amp; floor kit.</t>
+      </text>
+    </comment>
+    <comment ref="B90" authorId="0" shapeId="0">
+      <text>
+        <t>Size per USCD listing: 30"W x 1-1/2"H x 12"D, wall cabinet accessory, ships assembled. SK version not verified.</t>
+      </text>
+    </comment>
+    <comment ref="B97" authorId="0" shapeId="0">
+      <text>
+        <t>Alias of row 360 (U1884244RS master, Tall / Utility Roll-Out Cabinet Kit). This is the full cabinet kit, not a rollout tray accessory. Same code and supplier, so ReplacementMasterCode left blank to avoid a self-reference on import.</t>
+      </text>
+    </comment>
+    <comment ref="B98" authorId="0" shapeId="0">
+      <text>
+        <t>Alias of row 362 (U1890244RS master, Tall / Utility Roll-Out Cabinet Kit). This is the full cabinet kit, not a rollout tray accessory. Same code and supplier, so ReplacementMasterCode left blank to avoid a self-reference on import.</t>
+      </text>
+    </comment>
+    <comment ref="B99" authorId="0" shapeId="0">
+      <text>
+        <t>Alias of row 364 (U1896244RS master, Tall / Utility Roll-Out Cabinet Kit). This is the full cabinet kit, not a rollout tray accessory. Same code and supplier, so ReplacementMasterCode left blank to avoid a self-reference on import.</t>
+      </text>
+    </comment>
+    <comment ref="B114" authorId="0" shapeId="0">
+      <text>
+        <t>Alias of row 610 (WMSSHELF master, Wall / Wall Microwave Shelf). Same code and supplier, so ReplacementMasterCode left blank to avoid a self-reference on import.</t>
+      </text>
+    </comment>
+    <comment ref="B189" authorId="0" shapeId="0">
+      <text>
+        <t>Drawer count depends on distributor. USCD B30 = 2 doors, 2 drawers, 1 shelf, but USCD is phasing B30 out in favor of B30S (single drawer), and B30 is not offered in Oxford or Edgeline lines. CS/SK versions not verified.</t>
+      </text>
+    </comment>
     <comment ref="B226" authorId="0" shapeId="0">
       <text>
         <t>Master code: BMW30. MB30 (SK, row 244) is the same 30" microwave base.</t>
@@ -205,9 +240,54 @@
         <t>Industry standard: 9-inch base cabinets never have drawers. Treat any 9" base as a tray base / full height, never a drawer base.</t>
       </text>
     </comment>
+    <comment ref="B232" authorId="0" shapeId="0">
+      <text>
+        <t>42" diagonal corner sink base: the front/side piece (DCSF42, row 234) and the bottom/floor piece (SBF4242, row 86) must be purchased together; DCFF42 (row 232) is the combined front &amp; floor kit.</t>
+      </text>
+    </comment>
+    <comment ref="B233" authorId="0" shapeId="0">
+      <text>
+        <t>Alias of row 256 (DCSB36 master, Diagonal Corner Sink Base). Same code and supplier, so ReplacementMasterCode was left blank to avoid a self-reference on import.</t>
+      </text>
+    </comment>
+    <comment ref="B234" authorId="0" shapeId="0">
+      <text>
+        <t>42" diagonal corner sink base: the front/side piece (DCSF42, row 234) and the bottom/floor piece (SBF4242, row 86) must be purchased together; DCFF42 (row 232) is the combined front &amp; floor kit.</t>
+      </text>
+    </comment>
+    <comment ref="B256" authorId="0" shapeId="0">
+      <text>
+        <t>Master entry for DCSB36 (Faircrest/CS 36" Diagonal Corner Sink Base, 36W x 24D x 34-1/2H, 1 door, L/R hinge chosen at order). Row 233 is an alias/duplicate listing of this same cabinet.</t>
+      </text>
+    </comment>
     <comment ref="B307" authorId="0" shapeId="0">
       <text>
         <t>Master code: SHM8. SHM (SK, row 306) is the same shoe moulding.</t>
+      </text>
+    </comment>
+    <comment ref="B360" authorId="0" shapeId="0">
+      <text>
+        <t>Master entry for U1884244RS (USCD two-door 18"W x 24"D utility cabinet kit, 2 fixed shelves + 4 rollout shelves). Row 97 is an alias/duplicate listing of this same item.</t>
+      </text>
+    </comment>
+    <comment ref="B362" authorId="0" shapeId="0">
+      <text>
+        <t>Master entry for U1890244RS (USCD two-door 18"W x 24"D utility cabinet kit, 2 fixed shelves + 4 rollout shelves). Row 98 is an alias/duplicate listing of this same item.</t>
+      </text>
+    </comment>
+    <comment ref="B364" authorId="0" shapeId="0">
+      <text>
+        <t>Master entry for U1896244RS (USCD two-door 18"W x 24"D utility cabinet kit, 2 fixed shelves + 4 rollout shelves). Row 99 is an alias/duplicate listing of this same item.</t>
+      </text>
+    </comment>
+    <comment ref="B382" authorId="0" shapeId="0">
+      <text>
+        <t>Designer option note (rows 382-403, Vanity Sink Base): drawer side (Left or Right) should be a customer-selectable option so customers can build their own vanity, rather than separate rows per drawer side. Existing DL/DR rows are kept as-is for now; no new column added.</t>
+      </text>
+    </comment>
+    <comment ref="B610" authorId="0" shapeId="0">
+      <text>
+        <t>Master entry for WMSSHELF (USCD wall microwave shelf, 26-1/2"W x 3/4"H x 17"D, fits the 30"W wall open cabinet). Row 114 is an alias/duplicate listing of this same item.</t>
       </text>
     </comment>
     <comment ref="B614" authorId="0" shapeId="0">
@@ -2069,7 +2149,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA 36" Blind Base Cabinet </t>
+          <t>ADA 36" Blind Base Cabinet</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -3419,7 +3499,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>SBF4242; SBF4242</t>
+          <t>SBF4242</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -3569,7 +3649,7 @@
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>Stem Glass Holder — 30" W; height/depth TBD</t>
+          <t>Stem Glass Holder — 30" W x 1-1/2" H x 12" D</t>
         </is>
       </c>
       <c r="G90" s="11" t="inlineStr">
@@ -7024,7 +7104,7 @@
       </c>
       <c r="F189" s="11" t="inlineStr">
         <is>
-          <t>30" W x 34-1/2" H x 24" D Base Cabinet — 2 Doors, 1 or 2 Drawers by distributor (see Brand Attributes); shelves TBD</t>
+          <t>30" W x 34-1/2" H x 24" D Base Cabinet — 2 Doors, 1 or 2 Drawers by distributor (see Brand Attributes); 1 shelf</t>
         </is>
       </c>
       <c r="G189" s="11" t="inlineStr">
@@ -8064,7 +8144,7 @@
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>BER33; ERB36</t>
+          <t>ERB36</t>
         </is>
       </c>
       <c r="E219" s="2" t="inlineStr">
@@ -8864,7 +8944,7 @@
       </c>
       <c r="F242" s="11" t="inlineStr">
         <is>
-          <t>Base Easy Reach Cabinet - 33""W x 34-1/2""H x 24""D -1D-1S</t>
+          <t>Base Easy Reach Cabinet - 33"W x 34-1/2"H x 24"D -1D-1S</t>
         </is>
       </c>
       <c r="G242" s="11" t="inlineStr">
@@ -8899,7 +8979,7 @@
       </c>
       <c r="F243" s="11" t="inlineStr">
         <is>
-          <t>Base Easy Reach Cabinet - 36""W x 34-1/2""H x 24""D -1D-1S</t>
+          <t>Base Easy Reach Cabinet - 36"W x 34-1/2"H x 24"D -1D-1S</t>
         </is>
       </c>
       <c r="G243" s="11" t="inlineStr">
@@ -9359,7 +9439,7 @@
       </c>
       <c r="F256" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">36" Corner Drawer Base Cabinet </t>
+          <t>36" Diagonal Corner Sink Base Cabinet</t>
         </is>
       </c>
       <c r="G256" s="11" t="inlineStr">
@@ -9369,7 +9449,7 @@
       </c>
       <c r="H256" s="11" t="inlineStr">
         <is>
-          <t>Corner Drawer Base</t>
+          <t>Diagonal Corner Sink Base</t>
         </is>
       </c>
     </row>
@@ -13761,7 +13841,7 @@
       </c>
       <c r="F382" s="2" t="inlineStr">
         <is>
-          <t>Vanity Combo - 30" W x 21" D x 34-1/2" H 1 door, 3 Drawers on Left</t>
+          <t>Vanity Sink Base - 30" W x 21" D x 34-1/2" H 1 door, 3 Drawers on Left</t>
         </is>
       </c>
       <c r="G382" s="11" t="inlineStr">
@@ -13796,7 +13876,7 @@
       </c>
       <c r="F383" s="2" t="inlineStr">
         <is>
-          <t>Vanity Combo - 30" W x 21" D x 34-1/2" H 1 door, 3 Drawers on Right</t>
+          <t>Vanity Sink Base - 30" W x 21" D x 34-1/2" H 1 door, 3 Drawers on Right</t>
         </is>
       </c>
       <c r="G383" s="11" t="inlineStr">
@@ -14181,7 +14261,7 @@
       </c>
       <c r="F394" s="11" t="inlineStr">
         <is>
-          <t>24" W x 34-1/2" H x 21" D Vanity Combo Base — Drawers Left: 2 Drawers, 1 Door</t>
+          <t>24" W x 34-1/2" H x 21" D Vanity Sink Base — Drawers Left: 2 Drawers, 1 Door</t>
         </is>
       </c>
       <c r="G394" s="11" t="inlineStr">
@@ -14216,7 +14296,7 @@
       </c>
       <c r="F395" s="11" t="inlineStr">
         <is>
-          <t>24" W x 34-1/2" H x 21" D Vanity Combo Base — Drawers Right: 2 Drawers, 1 Door</t>
+          <t>24" W x 34-1/2" H x 21" D Vanity Sink Base — Drawers Right: 2 Drawers, 1 Door</t>
         </is>
       </c>
       <c r="G395" s="11" t="inlineStr">
@@ -14321,7 +14401,7 @@
       </c>
       <c r="F398" s="11" t="inlineStr">
         <is>
-          <t>Combo Vanity with 2 Drawers on Left - 30"W X 34 1/2"H X 21"D - 1 Door - 1 Long False Drawer Face - Two Drawers on Left-Side</t>
+          <t>Vanity Sink Base with 2 Drawers on Left - 30"W X 34 1/2"H X 21"D - 1 Door - 1 Long False Drawer Face - Two Drawers on Left-Side</t>
         </is>
       </c>
       <c r="G398" s="11" t="inlineStr">
@@ -14356,7 +14436,7 @@
       </c>
       <c r="F399" s="11" t="inlineStr">
         <is>
-          <t>Combo Vanity with 2 Drawers on Right - 30"W X 34 1/2"H X 21"D - 1 Door - 1 Long False Drawer Face - Two Drawers on Right-Side</t>
+          <t>Vanity Sink Base with 2 Drawers on Right - 30"W X 34 1/2"H X 21"D - 1 Door - 1 Long False Drawer Face - Two Drawers on Right-Side</t>
         </is>
       </c>
       <c r="G399" s="11" t="inlineStr">
@@ -14391,7 +14471,7 @@
       </c>
       <c r="F400" s="11" t="inlineStr">
         <is>
-          <t>Vanity Sink Base - 33"W x 34 1/2" x 21"D - 1D, 3 Left DRW</t>
+          <t>Vanity Sink Base - 33"W x 34 1/2"H x 21"D - 1D, 3 Left DRW</t>
         </is>
       </c>
       <c r="G400" s="11" t="inlineStr">
@@ -14426,7 +14506,7 @@
       </c>
       <c r="F401" s="11" t="inlineStr">
         <is>
-          <t>Vanity Sink Base - 33"W x 34 1/2" x 21"D - 1D, 3 Right DRW</t>
+          <t>Vanity Sink Base - 33"W x 34 1/2"H x 21"D - 1D, 3 Right DRW</t>
         </is>
       </c>
       <c r="G401" s="11" t="inlineStr">
@@ -14461,7 +14541,7 @@
       </c>
       <c r="F402" s="11" t="inlineStr">
         <is>
-          <t>Vanity Sink Base - 33"W x 34 1/2" x 21"D - 1 False Front,1D, 2 Left DRW</t>
+          <t>Vanity Sink Base - 33"W x 34 1/2"H x 21"D - 1 False Front,1D, 2 Left DRW</t>
         </is>
       </c>
       <c r="G402" s="11" t="inlineStr">
@@ -14496,7 +14576,7 @@
       </c>
       <c r="F403" s="11" t="inlineStr">
         <is>
-          <t>Vanity Sink Base - 33"W x 34 1/2" x 21"D - 1 False Front,1D, 2 Right DRW</t>
+          <t>Vanity Sink Base - 33"W x 34 1/2"H x 21"D - 1 False Front,1D, 2 Right DRW</t>
         </is>
       </c>
       <c r="G403" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Replace the cabinet descriptions workbook with the Faircrest door-thickness correction.
Keep the same path and rerun the admin round-trip parser dry run against the updated sheet.

Co-authored-by: 7809tom-sys <7809tom-sys@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/distributor-connections/cabinet-descriptions-corrected-2026-10-26.xlsx
+++ b/data/distributor-connections/cabinet-descriptions-corrected-2026-10-26.xlsx
@@ -190,6 +190,21 @@
     <author>Grok Bot</author>
   </authors>
   <commentList>
+    <comment ref="B69" authorId="0" shapeId="0">
+      <text>
+        <t>Door thickness 1" per Faircrest dealer listing (CabinetryStock: Single Glass Diagonal Door (Plain Glass) 15"W x 30/36/42"H x 1"D). Within the 1" max standard set by Tom. Glass pane thickness itself not published by Faircrest.</t>
+      </text>
+    </comment>
+    <comment ref="B70" authorId="0" shapeId="0">
+      <text>
+        <t>Door thickness 1" per Faircrest dealer listing (CabinetryStock: Single Glass Diagonal Door (Plain Glass) 15"W x 30/36/42"H x 1"D). Within the 1" max standard set by Tom. Glass pane thickness itself not published by Faircrest.</t>
+      </text>
+    </comment>
+    <comment ref="B71" authorId="0" shapeId="0">
+      <text>
+        <t>Door thickness 1" per Faircrest dealer listing (CabinetryStock: Single Glass Diagonal Door (Plain Glass) 15"W x 30/36/42"H x 1"D). Within the 1" max standard set by Tom. Glass pane thickness itself not published by Faircrest.</t>
+      </text>
+    </comment>
     <comment ref="B86" authorId="0" shapeId="0">
       <text>
         <t>42" diagonal corner sink base: the front/side piece (DCSF42, row 234) and the bottom/floor piece (SBF4242, row 86) must be purchased together; DCFF42 (row 232) is the combined front &amp; floor kit.</t>
@@ -2914,7 +2929,7 @@
       </c>
       <c r="F69" s="11" t="inlineStr">
         <is>
-          <t>Plain Glass (PG) Door Only — 15" W x 30" H, thickness TBD; fits DCW2430 / WDC2430 diagonal corner wall</t>
+          <t>Plain Glass (PG) Door Only — 15" W x 30" H x 1" D; fits DCW2430 / WDC2430 diagonal corner wall</t>
         </is>
       </c>
       <c r="G69" s="11" t="inlineStr">
@@ -2949,7 +2964,7 @@
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>Plain Glass (PG) Door Only — 15" W x 36" H, thickness TBD; fits DCW2436 / WDC2436 diagonal corner wall</t>
+          <t>Plain Glass (PG) Door Only — 15" W x 36" H x 1" D; fits DCW2436 / WDC2436 diagonal corner wall</t>
         </is>
       </c>
       <c r="G70" s="11" t="inlineStr">
@@ -2984,7 +2999,7 @@
       </c>
       <c r="F71" s="11" t="inlineStr">
         <is>
-          <t>Plain Glass (PG) Door Only — 15" W x 42" H, thickness TBD; fits DCW2442 / WDC2442 diagonal corner wall</t>
+          <t>Plain Glass (PG) Door Only — 15" W x 42" H x 1" D; fits DCW2442 / WDC2442 diagonal corner wall</t>
         </is>
       </c>
       <c r="G71" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Apply the S2496 and SPW description corrections to the cabinet workbook.
Replace the sheet with the latest corrected file and keep the 617-row parser dry run.

Co-authored-by: 7809tom-sys <7809tom-sys@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/distributor-connections/cabinet-descriptions-corrected-2026-10-26.xlsx
+++ b/data/distributor-connections/cabinet-descriptions-corrected-2026-10-26.xlsx
@@ -11664,7 +11664,7 @@
       </c>
       <c r="F319" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shelf Board - 24"W x 96"H x 3/4"D </t>
+          <t>Shelf Board - 24"W x 96"H x 3/4"D</t>
         </is>
       </c>
       <c r="G319" s="2" t="inlineStr">
@@ -12040,7 +12040,7 @@
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>36" x 96" Stained Plywood</t>
+          <t>36" x 96" x 1/4" Stained Plywood</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Set the SPW description to the Faircrest stained plywood panel wording.
Replace the sheet with the final corrected file and keep the 617-row parser dry run.

Co-authored-by: 7809tom-sys <7809tom-sys@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/distributor-connections/cabinet-descriptions-corrected-2026-10-26.xlsx
+++ b/data/distributor-connections/cabinet-descriptions-corrected-2026-10-26.xlsx
@@ -280,6 +280,11 @@
         <t>Master code: SHM8. SHM (SK, row 306) is the same shoe moulding.</t>
       </text>
     </comment>
+    <comment ref="B330" authorId="0" shapeId="0">
+      <text>
+        <t>Faircrest SPW is a 1/4" stained plywood panel, 36"H x 96"W, finished one side, grain runs bottom to top, can be cut to size on install (Faircrest dealer listings: thewhiteshaker.com, rtacabinets365.com BC-SPW).</t>
+      </text>
+    </comment>
     <comment ref="B359" authorId="0" shapeId="0">
       <text>
         <t>Master entry for U1884244RS (USCD two-door 18"W x 24"D utility cabinet kit, 2 fixed shelves + 4 rollout shelves). Row 97 is an alias/duplicate listing of this same item.</t>
@@ -12040,7 +12045,7 @@
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>36" x 96" x 1/4" Stained Plywood</t>
+          <t>Stained Plywood Panel - 96"W x 36"H x 1/4"D</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">

</xml_diff>